<commit_message>
Refine study queue, retries, and muscle brief layout
</commit_message>
<xml_diff>
--- a/src/data/muscles.xlsx
+++ b/src/data/muscles.xlsx
@@ -40,40 +40,58 @@
     <t>Innervation</t>
   </si>
   <si>
+    <t>Longus colli</t>
+  </si>
+  <si>
+    <t>C3-T1 Vertebrae</t>
+  </si>
+  <si>
+    <t>C1-C6 vertebrae</t>
+  </si>
+  <si>
+    <t>Cervical flexion/stability</t>
+  </si>
+  <si>
     <t>Supraspinatus</t>
   </si>
   <si>
-    <t>Longus colli</t>
+    <t>Anterior rami of spinal nerves C2-C6</t>
   </si>
   <si>
     <t>Multifidus</t>
   </si>
   <si>
+    <t>Longus capitis</t>
+  </si>
+  <si>
+    <t>Sacrum/transverse processes</t>
+  </si>
+  <si>
     <t>Supraspinous fossa</t>
   </si>
   <si>
-    <t>C3-T1 Vertebrae</t>
-  </si>
-  <si>
-    <t>Sacrum/transverse processes</t>
+    <t>C3-C6 transverse processes</t>
+  </si>
+  <si>
+    <t>Spinous processes</t>
+  </si>
+  <si>
+    <t>Basilar occiput</t>
+  </si>
+  <si>
+    <t>Extension (bilateral) , Ipsi lateral flexion and contra rotation (unilateral)</t>
   </si>
   <si>
     <t xml:space="preserve">Greater tubercle of humerus </t>
   </si>
   <si>
-    <t>Spinous processes</t>
-  </si>
-  <si>
-    <t>Extension (bilateral) , Ipsi lateral flexion and contra rotation (unilateral)</t>
+    <t>Head/neck flexion</t>
   </si>
   <si>
     <t>Dorsal rami of spinal nerves</t>
   </si>
   <si>
-    <t>C1-C6 vertebrae</t>
-  </si>
-  <si>
-    <t>Cervical flexion/stability</t>
+    <t>Anterior rami of spinal nerves C1-C3</t>
   </si>
   <si>
     <t>Initiates Shoulder Abduction, stabilizes humeral  head</t>
@@ -82,235 +100,328 @@
     <t>Erector spinae</t>
   </si>
   <si>
-    <t>Anterior rami of spinal nerves C2-C6</t>
+    <t>Sternocleidomastoid</t>
   </si>
   <si>
     <t>Suprascapular nerve C5-C6</t>
   </si>
   <si>
+    <t>Manubrium of sternum, medial clavicle</t>
+  </si>
+  <si>
     <t>Iliac crest, sacrum</t>
   </si>
   <si>
+    <t>Infraspinatus</t>
+  </si>
+  <si>
+    <t>Mastoid process</t>
+  </si>
+  <si>
     <t>Ribs, vertebrae, skull</t>
   </si>
   <si>
-    <t>Longus capitis</t>
-  </si>
-  <si>
-    <t>Infraspinatus</t>
-  </si>
-  <si>
-    <t>C3-C6 transverse processes</t>
+    <t>Infraspinous fossa</t>
   </si>
   <si>
     <t>Extension (bilateral) , Ipsi lateral flexion (unilateral)</t>
   </si>
   <si>
-    <t>Infraspinous fossa</t>
-  </si>
-  <si>
-    <t>Basilar occiput</t>
+    <t xml:space="preserve">Flexion (bilateral) , contra rotation and ipsi sidebend (unilateral) </t>
+  </si>
+  <si>
+    <t>Spinal accessory (CN XI)</t>
   </si>
   <si>
     <t>Greater tubercle</t>
   </si>
   <si>
-    <t>Head/neck flexion</t>
+    <t>Rotatores</t>
+  </si>
+  <si>
+    <t>Scalenes</t>
   </si>
   <si>
     <t xml:space="preserve">Shoulder External rotation, stabilizes humeral head </t>
   </si>
   <si>
-    <t>Anterior rami of spinal nerves C1-C3</t>
-  </si>
-  <si>
-    <t>Rotatores</t>
-  </si>
-  <si>
     <t>Transverse processes</t>
   </si>
   <si>
-    <t>Sternocleidomastoid</t>
+    <t>C2-C7 transverse processes</t>
+  </si>
+  <si>
+    <t>Superior spinous processes</t>
+  </si>
+  <si>
+    <t>Ribs 1-2</t>
   </si>
   <si>
     <t>Teres minor</t>
   </si>
   <si>
-    <t>Superior spinous processes</t>
-  </si>
-  <si>
-    <t>Manubrium of sternum, medial clavicle</t>
+    <t xml:space="preserve">ipsi sidebending (unilateral)  , rib 1-2 elevation </t>
+  </si>
+  <si>
+    <t>Extension (bilateral), Contralateral rotation (unilateral)</t>
+  </si>
+  <si>
+    <t>Anterior rami of spinal nerves C3-C8</t>
   </si>
   <si>
     <t>Lateral scapula</t>
   </si>
   <si>
-    <t>Extension (bilateral), Contralateral rotation (unilateral)</t>
-  </si>
-  <si>
-    <t>Mastoid process</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flexion (bilateral) , contra rotation and ipsi sidebend (unilateral) </t>
+    <t>Biceps brachii</t>
+  </si>
+  <si>
+    <t>Quadratus lumborum</t>
+  </si>
+  <si>
+    <t>Levator scapulae</t>
+  </si>
+  <si>
+    <t>short head-coracoid process; long head- supraglenoid tubercle of scapula</t>
+  </si>
+  <si>
+    <t>Iliac crest</t>
+  </si>
+  <si>
+    <t>C1-C4 transverse processes</t>
+  </si>
+  <si>
+    <t>Radial tuberosity</t>
+  </si>
+  <si>
+    <t>12th rib, L1-L4</t>
+  </si>
+  <si>
+    <t>Superior medial scapula</t>
+  </si>
+  <si>
+    <t>Elbow flexion, supination</t>
+  </si>
+  <si>
+    <t>Extension (bilateral), Ipsilateral sidebend (unilateral)</t>
+  </si>
+  <si>
+    <t>cervical sidebend (ipsilateral); scapular evelation and downward rotation</t>
+  </si>
+  <si>
+    <t>Musculocutaneous nerve C5-C7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T12-L4 anterior rami spinal nerves </t>
+  </si>
+  <si>
+    <t>Anterior rami C3-C4 and dorsal scapular nerve (c5)</t>
+  </si>
+  <si>
+    <t>Brachialis</t>
+  </si>
+  <si>
+    <t>Suboccipitals</t>
+  </si>
+  <si>
+    <t>Distal Anterior humerus</t>
+  </si>
+  <si>
+    <t>Psoas major</t>
   </si>
   <si>
     <t>Axillary nerve C5-C6</t>
   </si>
   <si>
-    <t>Spinal accessory (CN XI)</t>
-  </si>
-  <si>
-    <t>Quadratus lumborum</t>
-  </si>
-  <si>
-    <t>Iliac crest</t>
+    <t>C1-C2</t>
+  </si>
+  <si>
+    <t>T12-L5 vertebrae</t>
+  </si>
+  <si>
+    <t>Coronoid process of ulna</t>
   </si>
   <si>
     <t>Subscapularis</t>
   </si>
   <si>
-    <t>Scalenes</t>
-  </si>
-  <si>
-    <t>12th rib, L1-L4</t>
+    <t>Lesser trochanter</t>
+  </si>
+  <si>
+    <t>Occiput and C1</t>
+  </si>
+  <si>
+    <t>Elbow flexion</t>
   </si>
   <si>
     <t>Subscapular fossa</t>
   </si>
   <si>
-    <t>C2-C7 transverse processes</t>
-  </si>
-  <si>
-    <t>Extension (bilateral), Ipsilateral sidebend (unilateral)</t>
+    <t>Hip flexion and slight ER , trunk sidebend (unilateral) trunk flexion (bilateral)</t>
+  </si>
+  <si>
+    <t>Musculocutaneous nerve C5-C6</t>
   </si>
   <si>
     <t>Lesser tubercle</t>
   </si>
   <si>
-    <t>Ribs 1-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T12-L4 anterior rami spinal nerves </t>
+    <t>L1-L3 anterior rami of spinal nerves</t>
   </si>
   <si>
     <t>Shoulder Internal rotation</t>
   </si>
   <si>
-    <t xml:space="preserve">ipsi sidebending (unilateral)  , rib 1-2 elevation </t>
+    <t>Transversus abdominis</t>
   </si>
   <si>
     <t>Upper and Lower Subscapular nerve C5-C7</t>
   </si>
   <si>
-    <t>Anterior rami of spinal nerves C3-C8</t>
-  </si>
-  <si>
-    <t>Psoas major</t>
-  </si>
-  <si>
-    <t>T12-L5 vertebrae</t>
+    <t>Brachioradialis</t>
+  </si>
+  <si>
+    <t>Thoracolumbar fascia, ribs</t>
+  </si>
+  <si>
+    <t>Lateral humerus</t>
+  </si>
+  <si>
+    <t>Linea alba</t>
+  </si>
+  <si>
+    <t>Distal radius</t>
   </si>
   <si>
     <t>Teres major</t>
   </si>
   <si>
-    <t>Levator scapulae</t>
-  </si>
-  <si>
-    <t>Lesser trochanter</t>
+    <t>Abdominal compression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elbow flexion </t>
   </si>
   <si>
     <t>Inferior angle of scapula</t>
   </si>
   <si>
-    <t>C1-C4 transverse processes</t>
-  </si>
-  <si>
-    <t>Hip flexion and slight ER , trunk sidebend (unilateral) trunk flexion (bilateral)</t>
+    <t xml:space="preserve">T7-L1 anterior rami of spinal nerves </t>
+  </si>
+  <si>
+    <t>Radial nerve C5-C7</t>
   </si>
   <si>
     <t>Intertubular sulcus (humerus)</t>
   </si>
   <si>
-    <t>Superior medial scapula</t>
-  </si>
-  <si>
-    <t>L1-L3 anterior rami of spinal nerves</t>
+    <t>Internal oblique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head extension, ipsilateral rotation </t>
+  </si>
+  <si>
+    <t>Triceps brachii</t>
   </si>
   <si>
     <t>Shoulder Extension, IR</t>
   </si>
   <si>
-    <t>cervical sidebend (ipsilateral); scapular evelation and downward rotation</t>
+    <t>Suboccipital nerve C1</t>
+  </si>
+  <si>
+    <t>LongHead- infraglenoid tubercle, Medial and Lateral head- posterior humerus</t>
   </si>
   <si>
     <t>Lower Subscapular Nerve (C5-C7)</t>
   </si>
   <si>
-    <t>Transversus abdominis</t>
-  </si>
-  <si>
-    <t>Anterior rami C3-C4 and dorsal scapular nerve (c5)</t>
+    <t>Semispinalis capitis</t>
+  </si>
+  <si>
+    <t>Olecranon process</t>
+  </si>
+  <si>
+    <t>Ribs 10-12, linea alba</t>
+  </si>
+  <si>
+    <t>C4-T6 transverse/articular processes</t>
+  </si>
+  <si>
+    <t>Elbow extension</t>
+  </si>
+  <si>
+    <t>Occiput</t>
+  </si>
+  <si>
+    <t>Trunk flexion (bilateral),  Ipsilateral rotation and sidebend (unilateral)</t>
   </si>
   <si>
     <t>Latissimus dorsi</t>
   </si>
   <si>
-    <t>Thoracolumbar fascia, ribs</t>
+    <t>Radial nerve C6-C8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6-L1 anterior rami of spinal nerves </t>
+  </si>
+  <si>
+    <t>Head extension (bilateral) , contralateral rotation/ ipsilateral sidebend (unilateral)</t>
   </si>
   <si>
     <t>T7-L5, iliac crest</t>
   </si>
   <si>
-    <t>Suboccipitals</t>
-  </si>
-  <si>
-    <t>Linea alba</t>
+    <t>Greater Occipital nerve C2 and C3 spinal nerve</t>
+  </si>
+  <si>
+    <t>Rectus abdominis</t>
   </si>
   <si>
     <t>Intertuberular sulcus of Humerus</t>
   </si>
   <si>
-    <t>C1-C2</t>
-  </si>
-  <si>
-    <t>Abdominal compression</t>
+    <t>Pubic crest</t>
   </si>
   <si>
     <t>Shoulder Extension, adduction, IR</t>
   </si>
   <si>
-    <t xml:space="preserve">T7-L1 anterior rami of spinal nerves </t>
+    <t>Xiphoid and ribs 5-7</t>
+  </si>
+  <si>
+    <t>Trunk flexion</t>
   </si>
   <si>
     <t>Thoracodorsal C6-C8</t>
   </si>
   <si>
-    <t>Internal oblique</t>
-  </si>
-  <si>
-    <t>Caracobrachialis</t>
+    <t xml:space="preserve">T6-T12 anterior rami of spinal nerves </t>
+  </si>
+  <si>
+    <t>Anconeus</t>
+  </si>
+  <si>
+    <t>Coracobrachialis</t>
+  </si>
+  <si>
+    <t>External oblique</t>
+  </si>
+  <si>
+    <t>External surface ribs 5-12</t>
+  </si>
+  <si>
+    <t>pubic tubercle, linea alba, anterior half of iliac crest</t>
   </si>
   <si>
     <t>Coracoid Process</t>
   </si>
   <si>
-    <t>Occiput and C1</t>
-  </si>
-  <si>
-    <t>Ribs 10-12, linea alba</t>
+    <t>Trunk flexion (bilateral),  Contra rotation and Ipsi sidebend (unilateral)</t>
   </si>
   <si>
     <t>Anteromedial surface of humerus</t>
   </si>
   <si>
-    <t xml:space="preserve">Head extension, ipsilateral rotation </t>
-  </si>
-  <si>
-    <t>Trunk flexion (bilateral),  Ipsilateral rotation and sidebend (unilateral)</t>
-  </si>
-  <si>
-    <t>Suboccipital nerve C1</t>
+    <t xml:space="preserve">T7-T12 anterior rami of spinal nerves </t>
   </si>
   <si>
     <t>Shoulder flexion/adduction</t>
@@ -319,55 +430,46 @@
     <t>Musculocutaneous nerve (C5-C7)</t>
   </si>
   <si>
-    <t>Semispinalis capitis</t>
+    <t>Lateral epicondyle of humerus</t>
   </si>
   <si>
     <t>Deltoid</t>
   </si>
   <si>
-    <t>C4-T6 transverse/articular processes</t>
+    <t>Lateral surface of Olecranon</t>
   </si>
   <si>
     <t>Clavicle/acromion/scapular spine</t>
   </si>
   <si>
-    <t xml:space="preserve">T6-L1 anterior rami of spinal nerves </t>
-  </si>
-  <si>
-    <t>Occiput</t>
+    <t>Elbow extension/stabilization</t>
   </si>
   <si>
     <t>Deltoid tuberosity</t>
   </si>
   <si>
+    <t>Radial Nerve C7-C8</t>
+  </si>
+  <si>
     <t>Shoulder Flexion, abduction, extension</t>
   </si>
   <si>
-    <t>Head extension (bilateral) , contralateral rotation/ ipsilateral sidebend (unilateral)</t>
-  </si>
-  <si>
-    <t>Rectus abdominis</t>
-  </si>
-  <si>
-    <t>Pubic crest</t>
-  </si>
-  <si>
-    <t>Greater Occipital nerve C2 and C3 spinal nerve</t>
-  </si>
-  <si>
-    <t>Xiphoid and ribs 5-7</t>
+    <t>Supinator</t>
   </si>
   <si>
     <t>Pectoralis major</t>
   </si>
   <si>
-    <t>Trunk flexion</t>
+    <t>Proximal Radius</t>
   </si>
   <si>
     <t>Clavicle/sternum</t>
   </si>
   <si>
-    <t xml:space="preserve">T6-T12 anterior rami of spinal nerves </t>
+    <t>Supination</t>
+  </si>
+  <si>
+    <t>Deep radial nerve C6-C7</t>
   </si>
   <si>
     <t>Latereral Intertubercular sulcus of Humerus</t>
@@ -376,45 +478,57 @@
     <t>Shoulder Flexion, adduction, IR</t>
   </si>
   <si>
-    <t>External oblique</t>
+    <t xml:space="preserve">Pronator Quadratus </t>
   </si>
   <si>
     <t>Lateral Pectoral nerve and medial pectoral nerve  C5-T1</t>
   </si>
   <si>
-    <t>External surface ribs 5-12</t>
-  </si>
-  <si>
-    <t>pubic tubercle, linea alba, anterior half of iliac crest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pectoral minor </t>
-  </si>
-  <si>
-    <t>Trunk flexion (bilateral),  Contra rotation and Ipsi sidebend (unilateral)</t>
+    <t xml:space="preserve">Pronator ridge (anterior distal ulna) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pectoralis minor </t>
   </si>
   <si>
     <t>Sternal end of ribs 3-5</t>
   </si>
   <si>
-    <t xml:space="preserve">T7-T12 anterior rami of spinal nerves </t>
+    <t xml:space="preserve">Anterior distal radius </t>
+  </si>
+  <si>
+    <t>Pronation</t>
   </si>
   <si>
     <t>Stabilizes scapula, scapular protraction/depression</t>
   </si>
   <si>
+    <t>Anterior Interosseus nerve C7-T1</t>
+  </si>
+  <si>
     <t>Medial Pectoral nerve (C8-T1)</t>
   </si>
   <si>
+    <t>Pronator teres</t>
+  </si>
+  <si>
     <t>Serratus anterior</t>
   </si>
   <si>
+    <t>Medial epicondyle (humeral head) ; coronoid process of ulna (ulnar head)</t>
+  </si>
+  <si>
+    <t>Pronator Tuberosity of Radius</t>
+  </si>
+  <si>
     <t>Ribs 1-8</t>
   </si>
   <si>
     <t>Medial scapula</t>
   </si>
   <si>
+    <t>Median nerve C6-C7</t>
+  </si>
+  <si>
     <t>Scapular Protraction/upward rotation</t>
   </si>
   <si>
@@ -478,120 +592,6 @@
     <t>Spinal accessory nerve (CN XI) and spinal nerves C3-C4</t>
   </si>
   <si>
-    <t>Biceps brachii</t>
-  </si>
-  <si>
-    <t>short head-coracoid process; long head- supraglenoid tubercle of scapula</t>
-  </si>
-  <si>
-    <t>Radial tuberosity</t>
-  </si>
-  <si>
-    <t>Elbow flexion, supination</t>
-  </si>
-  <si>
-    <t>Musculocutaneous nerve C5-C7</t>
-  </si>
-  <si>
-    <t>Brachialis</t>
-  </si>
-  <si>
-    <t>Distal Anterior humerus</t>
-  </si>
-  <si>
-    <t>Coronoid process of ulna</t>
-  </si>
-  <si>
-    <t>Elbow flexion</t>
-  </si>
-  <si>
-    <t>Musculocutaneous nerve C5-C6</t>
-  </si>
-  <si>
-    <t>Brachioradialis</t>
-  </si>
-  <si>
-    <t>Lateral humerus</t>
-  </si>
-  <si>
-    <t>Distal radius</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elbow flexion </t>
-  </si>
-  <si>
-    <t>Radial nerve C5-C7</t>
-  </si>
-  <si>
-    <t>Triceps brachii</t>
-  </si>
-  <si>
-    <t>LongHead- infraglenoid tubercle, Medial and Lateral head- posterior humerus</t>
-  </si>
-  <si>
-    <t>Olecranon process</t>
-  </si>
-  <si>
-    <t>Elbow extension</t>
-  </si>
-  <si>
-    <t>Radial nerve C6-C8</t>
-  </si>
-  <si>
-    <t>Anconeus</t>
-  </si>
-  <si>
-    <t>Lateral epicondyle of humerus</t>
-  </si>
-  <si>
-    <t>Lateral surface of Olecranon</t>
-  </si>
-  <si>
-    <t>Elbow extension/stabilization</t>
-  </si>
-  <si>
-    <t>Radial Nerve C7-C8</t>
-  </si>
-  <si>
-    <t>Supinator</t>
-  </si>
-  <si>
-    <t>Proximal Radius</t>
-  </si>
-  <si>
-    <t>Supination</t>
-  </si>
-  <si>
-    <t>Deep radial nerve C6-C7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pronator Quadratus </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pronator ridge (anterior distal ulna) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anterior distal radius </t>
-  </si>
-  <si>
-    <t>Pronation</t>
-  </si>
-  <si>
-    <t>Anterior Interosseus nerve C7-T1</t>
-  </si>
-  <si>
-    <t>Pronator teres</t>
-  </si>
-  <si>
-    <t>Medial epicondyle (humeral head) ; coronoid process of ulna (ulnar head)</t>
-  </si>
-  <si>
-    <t>Pronator Tuberosity of Radius</t>
-  </si>
-  <si>
-    <t>Median nerve C6-C7</t>
-  </si>
-  <si>
     <t>Flexor carpi radialis</t>
   </si>
   <si>
@@ -604,526 +604,526 @@
     <t xml:space="preserve">Wrist flexion, radial deviation </t>
   </si>
   <si>
+    <t>Flexor carpi ulnaris</t>
+  </si>
+  <si>
+    <t>Medial epicondyle/ulna</t>
+  </si>
+  <si>
+    <t>Pisiform</t>
+  </si>
+  <si>
+    <t>Wrist flexion, ulnar deviation</t>
+  </si>
+  <si>
+    <t>Ulnar nerve C7-T1</t>
+  </si>
+  <si>
+    <t>Extensor carpi ulnaris</t>
+  </si>
+  <si>
+    <t>Lateral epicondyle</t>
+  </si>
+  <si>
+    <t>Base of 5th metacarpal</t>
+  </si>
+  <si>
+    <t>Wrist extension, ulnar deviation</t>
+  </si>
+  <si>
+    <t>Posterior interosseous nerve (deep branch of radial) C7-C8</t>
+  </si>
+  <si>
+    <t>Extensor carpi radialis longus</t>
+  </si>
+  <si>
+    <t>Lateral supracondylar ridge</t>
+  </si>
+  <si>
+    <t>base of 2nd metacarpal</t>
+  </si>
+  <si>
+    <t>Wrist extension</t>
+  </si>
+  <si>
+    <t>Radial nerve C6-C7</t>
+  </si>
+  <si>
+    <t>Extensor Carpi Radialis Brevis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">base of 3rd metacarpal </t>
+  </si>
+  <si>
+    <t>Wrist extension and radial deviation</t>
+  </si>
+  <si>
+    <t>Radial nerve (C5-C6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extensor Digitorum </t>
+  </si>
+  <si>
+    <t>Extensor expansions digits 2-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extends fingers 2-5 (assists wrist extension) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posterior Interosseus nerve (C7-C8) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extensor Pollicis Longus </t>
+  </si>
+  <si>
+    <t>Gluteus maximus</t>
+  </si>
+  <si>
+    <t>Posterior ulna and interosseus membrane</t>
+  </si>
+  <si>
+    <t>posterior Ilium/sacrum/coccyx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distal phalanx of thum </t>
+  </si>
+  <si>
+    <t>IT band, femur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extends thumb IP, MCP, CMC </t>
+  </si>
+  <si>
+    <t>Hip extension</t>
+  </si>
+  <si>
+    <t>Inferior gluteal nerve L5-S2</t>
+  </si>
+  <si>
+    <t>Extensor Pollicis Brevis</t>
+  </si>
+  <si>
+    <t>Gluteus medius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posterior distal radius </t>
+  </si>
+  <si>
+    <t>external surface of ilium between anterior and posterior gluteal lines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posterior base of proximal phalanx of thumb </t>
+  </si>
+  <si>
+    <t>Greater trochanter</t>
+  </si>
+  <si>
+    <t>Hip abduction</t>
+  </si>
+  <si>
+    <t>Thumb MCP and CMC extension</t>
+  </si>
+  <si>
+    <t>Superior gluteal nerve L4-S1</t>
+  </si>
+  <si>
+    <t>Posterior Interosseus nerve (C7-C8)</t>
+  </si>
+  <si>
+    <t>Gluteus minimus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abductor Pollicis Longus </t>
+  </si>
+  <si>
+    <t>external surface of ilium between anterior and inferior gluteal lines</t>
+  </si>
+  <si>
+    <t>Posterior radius and ulna, interosseus membrane</t>
+  </si>
+  <si>
+    <t>Base of 1st metacarpal</t>
+  </si>
+  <si>
+    <t>Hip abduction, IR</t>
+  </si>
+  <si>
+    <t>Thumb CMC abduction and extension</t>
+  </si>
+  <si>
+    <t>Tensor fasciae latae</t>
+  </si>
+  <si>
+    <t>Flexor digitorum superficialis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anterior Superior Iliac Spine </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medial epicondyle, coronoud process of ulna, proximal anterior radius </t>
+  </si>
+  <si>
+    <t>IT band</t>
+  </si>
+  <si>
+    <t>Middle phalanges</t>
+  </si>
+  <si>
+    <t>Hip flexion/abduction</t>
+  </si>
+  <si>
+    <t>Finger flexion</t>
+  </si>
+  <si>
+    <t>Median C7-T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flexor Digitorum Profundus </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rectus Femoris </t>
+  </si>
+  <si>
+    <t>Anterior Superior Iliac Spine and superior acetabular rim</t>
+  </si>
+  <si>
+    <t>Tibial tuberosity via patellar tendon</t>
+  </si>
+  <si>
+    <t>Hip flexion, knee extension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Femoral nerve L2-L4 </t>
+  </si>
+  <si>
+    <t>Proximal anterior and medial ulna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distal phalanges 2-5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartorius </t>
+  </si>
+  <si>
+    <t>Flexes DIP joints (assist wrist flexion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lateral half (median);Medial half (Ulnar) C8-T1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pes anserine </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flexor Pollicis Longus </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hip abduction, flexion, external rotation; knee flexion </t>
+  </si>
+  <si>
+    <t>Anterior radius and interosseus membrane</t>
+  </si>
+  <si>
+    <t>Femoral nerve L2-L3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distal phalanx of thumb </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flexes thumb IP joints </t>
+  </si>
+  <si>
+    <t>Piriformis</t>
+  </si>
+  <si>
+    <t>Anterior Interosseus nerve (C8-T1)</t>
+  </si>
+  <si>
+    <t>Interossei</t>
+  </si>
+  <si>
+    <t>Anterior Sacrum</t>
+  </si>
+  <si>
+    <t>Adjacent metacarpals</t>
+  </si>
+  <si>
+    <t>Greater trochanter (superior border)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proximal phalanges </t>
+  </si>
+  <si>
+    <t>Hip ER,</t>
+  </si>
+  <si>
+    <t>nerve to piriformis S1-S2</t>
+  </si>
+  <si>
+    <t>Dorsal-finger abduction Palmar- finger adduction</t>
+  </si>
+  <si>
+    <t>Ulnar nerve C8-T1)</t>
+  </si>
+  <si>
+    <t>Adductor Longus</t>
+  </si>
+  <si>
+    <t>Body of Pubis inferior to pubic crest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opponens Pollicis </t>
+  </si>
+  <si>
+    <t>Flexor retinaculum and trapezium</t>
+  </si>
+  <si>
+    <t>Medial third linea aspera</t>
+  </si>
+  <si>
+    <t>Lateral shaft of 1st metacarpal</t>
+  </si>
+  <si>
+    <t>Opposition of thumb</t>
+  </si>
+  <si>
+    <t>Hip adduction, assists flexion</t>
+  </si>
+  <si>
+    <t>Median nerve (C8-T1)</t>
+  </si>
+  <si>
+    <t>Obturator Nerve L2-L4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumbricals </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adductor Magus </t>
+  </si>
+  <si>
+    <t>Tendons of flexor digitorum profundus</t>
+  </si>
+  <si>
+    <t>Inferior Pubic ramus, ischial ramus, ischial tuberosity</t>
+  </si>
+  <si>
+    <t>Extensor expansion of digits 2-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linea aspera and adductor tubercle </t>
+  </si>
+  <si>
+    <t>MCP flexion and IP extension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hip adduction </t>
+  </si>
+  <si>
+    <t>Lumbricals 1-2 Median nerve ; Lumbricals 3-4 Ulnar nerve (C8-T1)</t>
+  </si>
+  <si>
+    <t>Obturator nerve L2-L4; Sciatic nerve L4-S1</t>
+  </si>
+  <si>
+    <t>Adductor Brevis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inferior Pubic ramus </t>
+  </si>
+  <si>
+    <t>Proximal linea aspera</t>
+  </si>
+  <si>
+    <t>Obturator nerve L2-L4</t>
+  </si>
+  <si>
+    <t>Biceps Femoris (long head)</t>
+  </si>
+  <si>
     <t>Rectus femoris</t>
   </si>
   <si>
+    <t xml:space="preserve">Ischial tuberosity </t>
+  </si>
+  <si>
     <t>AIIS (anterior inferior iliac spine)</t>
   </si>
   <si>
+    <t xml:space="preserve">head of fibula </t>
+  </si>
+  <si>
     <t>Tibial tuberosity via patella tendon</t>
   </si>
   <si>
-    <t>Flexor carpi ulnaris</t>
-  </si>
-  <si>
-    <t>Gluteus maximus</t>
+    <t>Hip extension, knee flexion</t>
   </si>
   <si>
     <t>Knee extension, hip flexion</t>
   </si>
   <si>
-    <t>Medial epicondyle/ulna</t>
+    <t xml:space="preserve">Tibial nerve L5-S2 </t>
   </si>
   <si>
     <t>Femoral nerve L2-L4</t>
   </si>
   <si>
-    <t>posterior Ilium/sacrum/coccyx</t>
-  </si>
-  <si>
-    <t>Pisiform</t>
-  </si>
-  <si>
-    <t>IT band, femur</t>
-  </si>
-  <si>
-    <t>Wrist flexion, ulnar deviation</t>
-  </si>
-  <si>
     <t>Vastus medialis</t>
   </si>
   <si>
-    <t>Hip extension</t>
-  </si>
-  <si>
-    <t>Ulnar nerve C7-T1</t>
+    <t xml:space="preserve">Semitendonosis </t>
   </si>
   <si>
     <t>Medial femur</t>
   </si>
   <si>
-    <t>Inferior gluteal nerve L5-S2</t>
-  </si>
-  <si>
     <t>Patella</t>
   </si>
   <si>
-    <t>Extensor carpi ulnaris</t>
-  </si>
-  <si>
     <t>Knee extension</t>
   </si>
   <si>
-    <t>Gluteus medius</t>
-  </si>
-  <si>
-    <t>Lateral epicondyle</t>
-  </si>
-  <si>
-    <t>external surface of ilium between anterior and posterior gluteal lines</t>
-  </si>
-  <si>
-    <t>Base of 5th metacarpal</t>
-  </si>
-  <si>
-    <t>Greater trochanter</t>
-  </si>
-  <si>
     <t>Vastus lateralis</t>
   </si>
   <si>
-    <t>Wrist extension, ulnar deviation</t>
-  </si>
-  <si>
-    <t>Hip abduction</t>
+    <t>Semimembranosus</t>
   </si>
   <si>
     <t>lateral femur</t>
   </si>
   <si>
-    <t>Posterior interosseous nerve (deep branch of radial) C7-C8</t>
-  </si>
-  <si>
-    <t>Superior gluteal nerve L4-S1</t>
-  </si>
-  <si>
-    <t>Extensor carpi radialis longus</t>
-  </si>
-  <si>
-    <t>Lateral supracondylar ridge</t>
-  </si>
-  <si>
-    <t>base of 2nd metacarpal</t>
+    <t xml:space="preserve">Posterior medial condyle of tibia </t>
   </si>
   <si>
     <t>Vastus Intermedialis</t>
   </si>
   <si>
-    <t>Gluteus minimus</t>
-  </si>
-  <si>
-    <t>Wrist extension</t>
-  </si>
-  <si>
     <t>Intertrochanteric line of femur</t>
   </si>
   <si>
-    <t>external surface of ilium between anterior and inferior gluteal lines</t>
-  </si>
-  <si>
-    <t>Radial nerve C6-C7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Patella </t>
   </si>
   <si>
-    <t>Hip abduction, IR</t>
-  </si>
-  <si>
     <t xml:space="preserve">Biceps femoris (short head) </t>
   </si>
   <si>
-    <t>Tensor fasciae latae</t>
-  </si>
-  <si>
     <t>Ischial tuberosity/femur</t>
   </si>
   <si>
-    <t xml:space="preserve">Anterior Superior Iliac Spine </t>
-  </si>
-  <si>
     <t>Fibular head</t>
   </si>
   <si>
-    <t>IT band</t>
-  </si>
-  <si>
     <t>Knee flexion</t>
   </si>
   <si>
-    <t>Hip flexion/abduction</t>
-  </si>
-  <si>
     <t>Common fibular nerve L5-S2</t>
   </si>
   <si>
-    <t xml:space="preserve">Rectus Femoris </t>
-  </si>
-  <si>
-    <t>Anterior Superior Iliac Spine and superior acetabular rim</t>
-  </si>
-  <si>
     <t>Semitendinosus</t>
   </si>
   <si>
-    <t>Extensor Carpi Radialis Brevis</t>
-  </si>
-  <si>
-    <t>Tibial tuberosity via patellar tendon</t>
-  </si>
-  <si>
     <t>Ischial tuberosity</t>
   </si>
   <si>
-    <t>Hip flexion, knee extension</t>
-  </si>
-  <si>
     <t>Pes anserine</t>
   </si>
   <si>
-    <t xml:space="preserve">Femoral nerve L2-L4 </t>
-  </si>
-  <si>
     <t>Knee flexion, hip extension</t>
   </si>
   <si>
-    <t xml:space="preserve">base of 3rd metacarpal </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tibial nerve L5-S2 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sartorius </t>
-  </si>
-  <si>
-    <t>Wrist extension and radial deviation</t>
-  </si>
-  <si>
-    <t>Semimembranosus</t>
-  </si>
-  <si>
-    <t>Radial nerve (C5-C6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pes anserine </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ischial tuberosity </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hip abduction, flexion, external rotation; knee flexion </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Posterior medial condyle of tibia </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extensor Digitorum </t>
-  </si>
-  <si>
-    <t>Femoral nerve L2-L3</t>
+    <t>Psoas Major</t>
+  </si>
+  <si>
+    <t>T12-L5 vertebral bodies, discs, and vertebral processes</t>
   </si>
   <si>
     <t>knee flexion, hip extension</t>
   </si>
   <si>
-    <t>Extensor expansions digits 2-5</t>
-  </si>
-  <si>
-    <t>Piriformis</t>
+    <t>Lesser trochanter of femur</t>
+  </si>
+  <si>
+    <t>Hip flexion, assists trunk flexion</t>
   </si>
   <si>
     <t>Gracilis</t>
   </si>
   <si>
-    <t xml:space="preserve">Extends fingers 2-5 (assists wrist extension) </t>
-  </si>
-  <si>
-    <t>Anterior Sacrum</t>
-  </si>
-  <si>
     <t>Body and inferior ramus of pubis</t>
   </si>
   <si>
-    <t xml:space="preserve">Posterior Interosseus nerve (C7-C8) </t>
-  </si>
-  <si>
-    <t>Greater trochanter (superior border)</t>
-  </si>
-  <si>
-    <t>Hip ER,</t>
-  </si>
-  <si>
     <t>Knee flexion, tibial IR; assists hip adduction</t>
   </si>
   <si>
-    <t>nerve to piriformis S1-S2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extensor Pollicis Longus </t>
-  </si>
-  <si>
     <t>Obturator nerve L2-L3</t>
   </si>
   <si>
-    <t>Posterior ulna and interosseus membrane</t>
-  </si>
-  <si>
-    <t>Adductor Longus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distal phalanx of thum </t>
-  </si>
-  <si>
     <t>Popliteus</t>
   </si>
   <si>
-    <t>Body of Pubis inferior to pubic crest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extends thumb IP, MCP, CMC </t>
-  </si>
-  <si>
     <t xml:space="preserve">Lateral femoral condyle, lateral meniscus </t>
   </si>
   <si>
-    <t>Medial third linea aspera</t>
-  </si>
-  <si>
     <t>Posterior proximal tibia</t>
   </si>
   <si>
-    <t>Hip adduction, assists flexion</t>
-  </si>
-  <si>
     <t>Tibal IR ,unlocks knee</t>
   </si>
   <si>
-    <t>Obturator Nerve L2-L4</t>
-  </si>
-  <si>
     <t>Tibial nerve L4-S1</t>
   </si>
   <si>
-    <t>Extensor Pollicis Brevis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Posterior distal radius </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adductor Magus </t>
-  </si>
-  <si>
-    <t>Inferior Pubic ramus, ischial ramus, ischial tuberosity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Posterior base of proximal phalanx of thumb </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linea aspera and adductor tubercle </t>
-  </si>
-  <si>
-    <t>Thumb MCP and CMC extension</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hip adduction </t>
-  </si>
-  <si>
-    <t>Posterior Interosseus nerve (C7-C8)</t>
-  </si>
-  <si>
-    <t>Obturator nerve L2-L4; Sciatic nerve L4-S1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abductor Pollicis Longus </t>
-  </si>
-  <si>
-    <t>Adductor Brevis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inferior Pubic ramus </t>
-  </si>
-  <si>
-    <t>Posterior radius and ulna, interosseus membrane</t>
-  </si>
-  <si>
-    <t>Proximal linea aspera</t>
-  </si>
-  <si>
-    <t>Base of 1st metacarpal</t>
-  </si>
-  <si>
-    <t>Thumb CMC abduction and extension</t>
-  </si>
-  <si>
-    <t>Obturator nerve L2-L4</t>
-  </si>
-  <si>
-    <t>Biceps Femoris (long head)</t>
-  </si>
-  <si>
-    <t>Flexor digitorum superficialis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medial epicondyle, coronoud process of ulna, proximal anterior radius </t>
-  </si>
-  <si>
-    <t xml:space="preserve">head of fibula </t>
-  </si>
-  <si>
-    <t>Middle phalanges</t>
-  </si>
-  <si>
-    <t>Hip extension, knee flexion</t>
-  </si>
-  <si>
-    <t>Finger flexion</t>
-  </si>
-  <si>
-    <t>Median C7-T1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semitendonosis </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flexor Digitorum Profundus </t>
-  </si>
-  <si>
-    <t>Proximal anterior and medial ulna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distal phalanges 2-5 </t>
-  </si>
-  <si>
-    <t>Flexes DIP joints (assist wrist flexion)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lateral half (median);Medial half (Ulnar) C8-T1 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flexor Pollicis Longus </t>
-  </si>
-  <si>
-    <t>Anterior radius and interosseus membrane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distal phalanx of thumb </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flexes thumb IP joints </t>
-  </si>
-  <si>
-    <t>Anterior Interosseus nerve (C8-T1)</t>
+    <t>Anterior rami L1-L3</t>
+  </si>
+  <si>
+    <t>Iliacus</t>
+  </si>
+  <si>
+    <t>Iliac fossa and iliac crest</t>
+  </si>
+  <si>
+    <t>Hip flexion, assists hip ER</t>
   </si>
   <si>
     <t>Gastrocnemius</t>
   </si>
   <si>
-    <t>Interossei</t>
-  </si>
-  <si>
-    <t>Psoas Major</t>
-  </si>
-  <si>
     <t>Medial and lateral condyles</t>
   </si>
   <si>
-    <t>Adjacent metacarpals</t>
-  </si>
-  <si>
-    <t>T12-L5 vertebral bodies, discs, and vertebral processes</t>
-  </si>
-  <si>
     <t>Posterior calcaneous</t>
   </si>
   <si>
-    <t xml:space="preserve">Proximal phalanges </t>
-  </si>
-  <si>
-    <t>Lesser trochanter of femur</t>
-  </si>
-  <si>
     <t>Ankle Plantarflexion, assists knee flexion</t>
   </si>
   <si>
-    <t>Dorsal-finger abduction Palmar- finger adduction</t>
-  </si>
-  <si>
-    <t>Hip flexion, assists trunk flexion</t>
-  </si>
-  <si>
     <t>Tibial nerve S1-S2</t>
   </si>
   <si>
-    <t>Ulnar nerve C8-T1)</t>
-  </si>
-  <si>
-    <t>Anterior rami L1-L3</t>
-  </si>
-  <si>
     <t>Soleus</t>
   </si>
   <si>
-    <t xml:space="preserve">Opponens Pollicis </t>
-  </si>
-  <si>
-    <t>Iliacus</t>
-  </si>
-  <si>
     <t>Posterior tibia and proximal fibula</t>
   </si>
   <si>
-    <t>Flexor retinaculum and trapezium</t>
-  </si>
-  <si>
-    <t>Iliac fossa and iliac crest</t>
-  </si>
-  <si>
     <t>Posterior calcaneus</t>
   </si>
   <si>
-    <t>Lateral shaft of 1st metacarpal</t>
-  </si>
-  <si>
     <t>Ankle Plantarflexion</t>
   </si>
   <si>
-    <t>Opposition of thumb</t>
-  </si>
-  <si>
-    <t>Hip flexion, assists hip ER</t>
-  </si>
-  <si>
-    <t>Median nerve (C8-T1)</t>
-  </si>
-  <si>
     <t>Tibialis anterior</t>
   </si>
   <si>
-    <t xml:space="preserve">Lumbricals </t>
-  </si>
-  <si>
     <t xml:space="preserve">Lateral tibia, lateral condyle of tibia </t>
   </si>
   <si>
-    <t>Tendons of flexor digitorum profundus</t>
-  </si>
-  <si>
     <t>Medial cuneiform and base of 1st Metatarsal</t>
   </si>
   <si>
-    <t>Extensor expansion of digits 2-5</t>
-  </si>
-  <si>
     <t>Dorsiflexion, inversion</t>
   </si>
   <si>
-    <t>MCP flexion and IP extension</t>
-  </si>
-  <si>
     <t>Deep fibular L4-L5</t>
-  </si>
-  <si>
-    <t>Lumbricals 1-2 Median nerve ; Lumbricals 3-4 Ulnar nerve (C8-T1)</t>
   </si>
   <si>
     <t>Tibialis posterior</t>
@@ -1545,121 +1545,121 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>9</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -2683,155 +2683,155 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3856,257 +3856,257 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>81</v>
+        <v>117</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>88</v>
+      <c r="A8" s="3" t="s">
+        <v>125</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>99</v>
+        <v>136</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>101</v>
+        <v>138</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>115</v>
+        <v>149</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>116</v>
+        <v>150</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>121</v>
+      <c r="A11" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>128</v>
+        <v>165</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>129</v>
+        <v>166</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>131</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>133</v>
+        <v>171</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>129</v>
+        <v>166</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>134</v>
+        <v>172</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>136</v>
+        <v>174</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>137</v>
+        <v>175</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>138</v>
+        <v>176</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>139</v>
+        <v>177</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>140</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>141</v>
+        <v>179</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>147</v>
+        <v>185</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>148</v>
+        <v>186</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>149</v>
+        <v>187</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5129,138 +5129,138 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>151</v>
+        <v>49</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>152</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>153</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>154</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>155</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>156</v>
+        <v>64</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>157</v>
+        <v>66</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>158</v>
+        <v>71</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>159</v>
+        <v>75</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>160</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>161</v>
+        <v>84</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>162</v>
+        <v>86</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>163</v>
+        <v>88</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>164</v>
+        <v>91</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>165</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>166</v>
+        <v>98</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>167</v>
+        <v>101</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>168</v>
+        <v>104</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>170</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>171</v>
+        <v>124</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>174</v>
+        <v>139</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>175</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>176</v>
+        <v>143</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>178</v>
+        <v>147</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>179</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>180</v>
+        <v>151</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>182</v>
+        <v>156</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>184</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -6297,245 +6297,245 @@
         <v>192</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>204</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>219</v>
+        <v>201</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>232</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>254</v>
+        <v>209</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>257</v>
+        <v>210</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>259</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>264</v>
+        <v>212</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>267</v>
+        <v>213</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>270</v>
+        <v>214</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>273</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>278</v>
+        <v>216</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>280</v>
+        <v>218</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>282</v>
+        <v>220</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>285</v>
+        <v>222</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>273</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>293</v>
+        <v>225</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>294</v>
+        <v>227</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>297</v>
+        <v>229</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>299</v>
+        <v>232</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>301</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>303</v>
+        <v>236</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>306</v>
+        <v>238</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>308</v>
+        <v>239</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>309</v>
+        <v>241</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>273</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>312</v>
+        <v>243</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>313</v>
+        <v>245</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>315</v>
+        <v>247</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>317</v>
+        <v>249</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>318</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>320</v>
+        <v>251</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>321</v>
+        <v>257</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>322</v>
+        <v>258</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>323</v>
+        <v>260</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>324</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>325</v>
+        <v>263</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>326</v>
+        <v>265</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>327</v>
+        <v>267</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>328</v>
+        <v>268</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>329</v>
+        <v>270</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>331</v>
+        <v>271</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>334</v>
+        <v>273</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>337</v>
+        <v>275</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>340</v>
+        <v>278</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>343</v>
+        <v>279</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>346</v>
+        <v>282</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>349</v>
+        <v>283</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>352</v>
+        <v>285</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>354</v>
+        <v>286</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>356</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>358</v>
+        <v>290</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>360</v>
+        <v>292</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>362</v>
+        <v>294</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>364</v>
+        <v>296</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>366</v>
+        <v>298</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -7560,118 +7560,118 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>221</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>274</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>277</v>
@@ -7679,138 +7679,138 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>258</v>
+        <v>320</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>263</v>
+        <v>322</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>338</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>338</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -8835,155 +8835,155 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>305</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>194</v>
+        <v>307</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>195</v>
+        <v>309</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>198</v>
+        <v>311</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>200</v>
+        <v>313</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>205</v>
+        <v>314</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>208</v>
+        <v>316</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>210</v>
+        <v>317</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>212</v>
+        <v>318</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>200</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>218</v>
+        <v>319</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>221</v>
+        <v>321</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>210</v>
+        <v>317</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>212</v>
+        <v>318</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>200</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>227</v>
+        <v>323</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>230</v>
+        <v>324</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>233</v>
+        <v>325</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>212</v>
+        <v>318</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>200</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>235</v>
+        <v>326</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>237</v>
+        <v>327</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>239</v>
+        <v>328</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>241</v>
+        <v>329</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>243</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>246</v>
+        <v>331</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>249</v>
+        <v>332</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>251</v>
+        <v>333</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>253</v>
+        <v>334</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>258</v>
+        <v>320</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>263</v>
+        <v>322</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>266</v>
+        <v>337</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>269</v>
+        <v>340</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>272</v>
+        <v>341</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>276</v>
+        <v>342</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>279</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>283</v>
+        <v>344</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>288</v>
+        <v>346</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>290</v>
+        <v>347</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>292</v>
+        <v>348</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -10008,53 +10008,53 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>330</v>
+        <v>353</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>333</v>
+        <v>354</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>339</v>
+        <v>356</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>348</v>
+        <v>359</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>351</v>
+        <v>360</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="5">
@@ -10127,7 +10127,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>264</v>
+        <v>212</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>387</v>
@@ -10167,7 +10167,7 @@
         <v>396</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>322</v>
+        <v>258</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>397</v>

</xml_diff>

<commit_message>
Add upper-extremity memory explanations and update muscle brief UI.
Correct shoulder and knee anatomy facts, add approved whyMemoryWorks content for upper-extremity profiles, show explanations directly in the muscle brief card, and include related memory illustration assets and tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/data/muscles.xlsx
+++ b/src/data/muscles.xlsx
@@ -716,7 +716,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1000"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -950,7 +950,7 @@
         <v xml:space="preserve">Lateral 1/3 of clavicle </v>
       </c>
       <c r="D14" t="str">
-        <v>Scapular retraction and downward rotation, shoulder girdle elevation</v>
+        <v>Scapular elevation and upward rotation</v>
       </c>
       <c r="E14" t="str">
         <v xml:space="preserve">Spinal Accessory Nerve (CN X1) and spinal nerves C3-C4 </v>
@@ -984,16 +984,15 @@
         <v>Lateral apex of medial scapular spine</v>
       </c>
       <c r="D16" t="str">
-        <v>Scapular Elevation/Retraction/Upward Rotation</v>
+        <v>Scapular depression, retraction, and upward rotation</v>
       </c>
       <c r="E16" t="str">
         <v>Spinal accessory nerve (CN XI) and spinal nerves C3-C4</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1000"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1681,7 +1680,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1000"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1770,7 +1769,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v xml:space="preserve">Biceps femoris (short head) </v>
+        <v>Biceps femoris</v>
       </c>
       <c r="B6" t="str">
         <v>Ischial tuberosity/femur</v>
@@ -1782,7 +1781,7 @@
         <v>Knee flexion</v>
       </c>
       <c r="E6" t="str">
-        <v>Common fibular nerve L5-S2</v>
+        <v>long head: tibial division of sciatic nerve (L5-S2) Short head: common fibular division of sciatic nerve (L5-S2)</v>
       </c>
     </row>
     <row r="7">
@@ -1799,7 +1798,7 @@
         <v>Knee flexion, hip extension</v>
       </c>
       <c r="E7" t="str">
-        <v xml:space="preserve">Tibial nerve L5-S2 </v>
+        <v>tibial division of sciatic nerve (L5-S2)</v>
       </c>
     </row>
     <row r="8">
@@ -1816,7 +1815,7 @@
         <v>knee flexion, hip extension</v>
       </c>
       <c r="E8" t="str">
-        <v xml:space="preserve">Tibial nerve L5-S2 </v>
+        <v>tibial division of sciatic nerve (L5-S2)</v>
       </c>
     </row>
     <row r="9">
@@ -1854,9 +1853,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1000"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix cervical data integrity and add lower extremity memory code
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/data/muscles.xlsx
+++ b/src/data/muscles.xlsx
@@ -428,7 +428,7 @@
         <v>Longus colli</v>
       </c>
       <c r="B2" t="str">
-        <v>C3-T1 Vertebrae</v>
+        <v>C3-T3</v>
       </c>
       <c r="C2" t="str">
         <v>C1-C6 vertebrae</v>
@@ -485,7 +485,7 @@
         <v>Ribs 1-2</v>
       </c>
       <c r="D5" t="str">
-        <v xml:space="preserve">ipsi sidebending (unilateral)  , rib 1-2 elevation </v>
+        <v>Neck flexion (bilateral), ipsilateral sidebend (unilateral), rib 1-2 elevation</v>
       </c>
       <c r="E5" t="str">
         <v>Anterior rami of spinal nerves C3-C8</v>
@@ -502,7 +502,7 @@
         <v>Superior medial scapula</v>
       </c>
       <c r="D6" t="str">
-        <v>cervical sidebend (ipsilateral); scapular evelation and downward rotation</v>
+        <v>Neck sidebend, elevation of the scapula, downward rotation of the scapula</v>
       </c>
       <c r="E6" t="str">
         <v>Anterior rami C3-C4 and dorsal scapular nerve (c5)</v>
@@ -530,16 +530,16 @@
         <v>Semispinalis capitis</v>
       </c>
       <c r="B8" t="str">
-        <v>C4-T6 transverse/articular processes</v>
+        <v>C4-T6 transverse and articular processes</v>
       </c>
       <c r="C8" t="str">
         <v>Occiput</v>
       </c>
       <c r="D8" t="str">
-        <v>Head extension (bilateral) , contralateral rotation/ ipsilateral sidebend (unilateral)</v>
+        <v>Head extension (bilateral), contralateral rotation and ipsilateral sidebend (unilateral)</v>
       </c>
       <c r="E8" t="str">
-        <v>Greater Occipital nerve C2 and C3 spinal nerve</v>
+        <v>Greater occipital nerve (C2) and C3 spinal nerve</v>
       </c>
     </row>
   </sheetData>

</xml_diff>